<commit_message>
added two more datasets for testing
</commit_message>
<xml_diff>
--- a/dataset_validation_tracker.xlsx
+++ b/dataset_validation_tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\home\hamza\dose_response_timepoint_selection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB78479-3D4D-460B-87EE-D0F02F38C000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D16E3F-6FE8-47AD-A01D-D8438FABA475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30612" yWindow="-1344" windowWidth="30936" windowHeight="16776" xr2:uid="{55B4DF3F-3158-4741-9A6E-3760371DC85B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t>Comment</t>
   </si>
@@ -71,15 +71,6 @@
     <t>https://github.com/NicWir/QurvE/blob/master/examples/custom_growth_2-FMA_toxicity.csv</t>
   </si>
   <si>
-    <t>custom_lac_promoters_od.csv</t>
-  </si>
-  <si>
-    <t>https://github.com/NicWir/QurvE/blob/master/examples/custom_lac_promoters.xlsx</t>
-  </si>
-  <si>
-    <t>OD sheet was taken out and reshaped</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -404,6 +395,116 @@
       </rPr>
       <t xml:space="preserve">16.95 to 17.05 </t>
     </r>
+  </si>
+  <si>
+    <t>https://github.com/tpetzoldt/growthrates/blob/master/data/bactgrowth.txt</t>
+  </si>
+  <si>
+    <t>converted to csv</t>
+  </si>
+  <si>
+    <t>bactgrowth</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">strain D: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>7.95 to 8.05</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>strain R:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 8.95 to 9.05</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">strain T: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>9.95 to 10.05</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">R: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6.45 to 6.55</t>
+    </r>
+  </si>
+  <si>
+    <t>antibiotic</t>
+  </si>
+  <si>
+    <t>converted to csv, made a fake column anibody to test the code</t>
+  </si>
+  <si>
+    <t>https://github.com/tpetzoldt/growthrates/blob/master/data/antibiotic.txt</t>
   </si>
 </sst>
 </file>
@@ -455,7 +556,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -478,12 +579,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -503,7 +641,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -844,7 +997,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD295D8-4683-435F-A0E9-260629365BB7}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultColWidth="34.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="1" bestFit="1" customWidth="1"/>
@@ -868,13 +1021,13 @@
         <v>0</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>1</v>
@@ -889,100 +1042,100 @@
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8">
+      <c r="A3" s="13">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="13"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G5" s="13"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="13"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="8"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="8"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="8"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>24</v>
-      </c>
       <c r="F7" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="G7" s="13"/>
     </row>
     <row r="8" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
@@ -992,13 +1145,13 @@
         <v>8</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="5" t="s">
@@ -1006,77 +1159,109 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="6">
+      <c r="A9" s="7">
         <v>4</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6" t="s">
-        <v>30</v>
+      <c r="B9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="F9" s="6"/>
-      <c r="G9" s="7" t="s">
-        <v>11</v>
+      <c r="G9" s="10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="8"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="11"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="12"/>
+    </row>
+    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
         <v>5</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="6">
+      <c r="B12" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="G12" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="6">
         <v>6</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
         <v>7</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C15" s="2"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C17" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="9">
     <mergeCell ref="G3:G7"/>
     <mergeCell ref="C3:C7"/>
     <mergeCell ref="B3:B7"/>
     <mergeCell ref="A3:A7"/>
+    <mergeCell ref="C9:C11"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="E9:E11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" xr:uid="{D6280971-B0FD-4C81-956A-4269FF3A684B}"/>
     <hyperlink ref="G8" r:id="rId2" xr:uid="{A231224D-ACCE-4AF1-AF0F-AF64F537A5CA}"/>
-    <hyperlink ref="G9" r:id="rId3" xr:uid="{497CFAC5-6BD7-4202-AD7F-2D18B99E0CF8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>